<commit_message>
feat: add topics column to article inventory Excel
</commit_message>
<xml_diff>
--- a/inventario-articulos-seo.xlsx
+++ b/inventario-articulos-seo.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00374151"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -85,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -95,6 +99,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -462,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -472,6 +479,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +518,11 @@
           <t>URL</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Puntos Tratados</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -545,6 +558,17 @@
           <t>https://apcvisionai.site/articulos/5-formas-analisis-flujo.html</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Análisis de flujo y zonas de calor
+• Conteo de personas para optimización de espacios
+• Mapas de calor para diseño de tiendas
+• Alertas de fila para equilibrio de personal
+• Analítica de eficiencia y KPIs operativos
+• Perspectiva integral de datos unificados
+• Implementación rápida en 72 horas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -580,6 +604,17 @@
           <t>https://apcvisionai.site/articulos/como-implementar-analisis-flujo.html</t>
         </is>
       </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Fase 1: exploración de requisitos y activos
+• Fase 2: planificación y cronograma
+• Fase 3: configuración técnica y desarrollo IA
+• Fase 4: prueba de usabilidad y validación
+• Dificultades comunes y soluciones
+• Consejos de implementación y checklist
+• Indicadores de éxito post-implementación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -615,6 +650,17 @@
           <t>https://apcvisionai.site/articulos/cuadres-de-caja-excel-ia.html</t>
         </is>
       </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Qué es un cuadre de caja y por qué falla
+• Por qué el cuadre manual en Excel no funciona
+• Cómo hacer cuadres con IA en 5 pasos
+• Plantilla Excel manual vs IA automatizada
+• Cuadre de caja diario como rutina de protección
+• IA para Excel: más allá del cuadre de caja
+• Caja registradora sistematizada con IA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -650,6 +696,17 @@
           <t>https://apcvisionai.site/articulos/arqueo-de-caja-excel.html</t>
         </is>
       </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Qué es el arqueo de caja
+• Problemas del arqueo manual en Excel
+• Automatizar arqueo con IA en 5 pasos
+• Plantilla manual vs Excel automatizado
+• Caja registradora sistematizada con IA
+• Cuadre de caja diario automatizado
+• IA para Excel: transcripción y búsqueda</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -685,6 +742,19 @@
           <t>https://apcvisionai.site/articulos/ia-para-excel-arqueo.html</t>
         </is>
       </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Qué es la IA para Excel
+• Por qué el Excel manual falla en arqueo
+• Captura automática de datos desde audio
+• Transcripción inteligente del conteo
+• Comparación POS vs conteo físico
+• Alertas automáticas por discrepancia
+• Reportes automáticos enviados por canal
+• Casos de uso reales: restaurante, retail, clínica
+• Calculadora de pérdida mensual</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -720,6 +790,16 @@
           <t>https://serviciosapc.site/blog/que-es-analitica-video-ia-empresas-bogota</t>
         </is>
       </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Qué es analítica de video con IA
+• Cómo funciona en 3 pasos (YOLO + Edge)
+• 7 casos de uso en empresas Bogotá
+• Por qué ahora: hardware compatible, YOLOv10
+• Mitos vs Realidad (cámaras, privacidad, internet)
+• Primer paso: auditoría gratis de cámaras</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -755,6 +835,18 @@
           <t>https://serviciosapc.site/blog/guia-camaras-hikvision-ia-empresas-bogota-2026</t>
         </is>
       </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Problema: cámaras vigilan pero no auditan
+• Qué es analítica de video YOLO
+• Compatibilidad con cámaras Hikvision existentes
+• Arquitectura Offline-First edge computing
+• Casos reales: ferretería, clínica, distribuidora
+• Modelos Hikvision recomendados 2026
+• Alertas en celular y dashboard
+• Integración n8n: CCTV a WhatsApp/CRM</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -790,6 +882,17 @@
           <t>https://serviciosapc.site/blog/costo-camaras-seguridad-empresas-2026-hardware-vs-ia</t>
         </is>
       </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>El mito de CCTV como gasto pasivo
+• Desglose real de costos: solo IA vs completa
+• Qué incluye la mensualidad de IA
+• ROI real con casos Bogotá
+• Costos ocultos que nadie te cuenta
+• Comparativa rápida: solo IA vs completa vs barata
+• Preguntas para cualquier proveedor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -825,6 +928,17 @@
           <t>https://serviciosapc.site/blog/5-senales-camaras-no-protegen-empresa-bogota</t>
         </is>
       </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Señal 1: cámara no grabó en momento clave
+• Señal 2: visión nocturna borrosa
+• Señal 3: puntos ciegos sin cobertura
+• Señal 4: arqueo de caja manual sin evidencia
+• Señal 5: técnico no contesta en emergencia
+• Checklist CCTV aprueba o reprueba
+• Plan de acción según número de señales</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -860,6 +974,17 @@
           <t>https://serviciosapc.site/blog/analitica-video-ia-ferreterias-bogota-caso-real-suba</t>
         </is>
       </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>El problema: ferretería como objetivo de robos
+• Solución: ColorVu 4K + IA YOLO
+• Qué detecta la IA en esta ferretería
+• Resultado 1: robo recuperado en 48h
+• Resultado 2: arqueo IA cero discrepancias
+• Resultado 3: mapa calor +18% ventas
+• ROI total: 324% en 5 meses</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -895,6 +1020,16 @@
           <t>https://serviciosapc.site/blog/negocio-camaras-ia-vs-sin-ia-caso-visual-antes-despues</t>
         </is>
       </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Tabla comparativa: antes vs después IA
+• Capturas reales del dashboard
+• Mapa de calor zona muerta detectada
+• Arqueo de caja IA reporte diario
+• Alertas reales WhatsApp/Telegram
+• ROI: ferretería El Progreso</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -930,6 +1065,16 @@
           <t>https://serviciosapc.site/blog/hikvision-colorvu-vs-acusense-vs-deepinview-ia-2026</t>
         </is>
       </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Tabla rápida: cuál necesito según prioridad
+• ColorVu: visión nocturna color real
+• AcuSense: mejor ROI filtro falsos positivos
+• DeepinView: IA embebida en cámara
+• Comparativa técnica completa 2026
+• Estrategia recomendada configuración ganadora</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -965,6 +1110,16 @@
           <t>https://serviciosapc.site/blog/analitica-video-ia-clinicas-bogota-cumplimiento-seguridad</t>
         </is>
       </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Reto único de clínicas en Bogotá
+• Arquitectura IA Offline-First para clínicas
+• 5 casos de uso: caídas, PPE, acceso, aforo, privacidad
+• Comparativa CCTV tradicional vs IA clínica
+• Caso real: Clínica Sonrisa Viva Chapinero
+• Inversión típica clínica 10-20 consultorios</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1000,6 +1155,17 @@
           <t>https://serviciosapc.site/blog/normativa-videovigilancia-colombia-2026-ley-1581-habeas-data</t>
         </is>
       </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Marco normativo 2026 CCTV en Colombia
+• Ley 1581 Habeas Data aplicada a CCTV+IA
+• Retención de video: qué dice la ley
+• Derechos ARCO en CCTV+IA
+• Resolución 1074 SG-SST y CCTV
+• Sanciones 2026 si no cumples
+• Checklist 20 items cumplimiento</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1035,6 +1201,16 @@
           <t>https://serviciosapc.site/blog/automatizacion-n8n-cctv-alerta-whatsapp-crm-dashboard</t>
         </is>
       </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Problema: cámaras graban pero no actúan
+• Qué es n8n y por qué cambia todo
+• Arquitectura: cámara a NVR a n8n a acción
+• Lógica condicional de alertas
+• Casos reales: ferretería, distribuidora, centro comercial
+• FAQ: self-hosted vs cloud, costos, soporte</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1070,6 +1246,18 @@
           <t>https://serviciosapc.site/blog/seo-local-google-maps-empresas-seguridad-bogota</t>
         </is>
       </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Problema: Google no te conoce
+• Qué es SEO Local y Google Business Profile
+• Optimizar GBP: categorías, descripción, fotos
+• Estrategia de reseñas y WhatsApp
+• Citas locales y directorios Bogotá
+• Keywords locales estratégicas
+• Contenido local por zona de servicio
+• Caso real: Distribuidora Jone +340%</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1105,6 +1293,17 @@
           <t>https://serviciosapc.site/blog/servidores-edge-gpu-para-ia-video-analitica-bogota</t>
         </is>
       </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Problema: costos de cloud para videoanalítica
+• Edge computing para videoanalítica
+• Arquitectura edge completa diagrama
+• Requisitos del servidor edge GPU
+• Comparativa GPUs: T4 vs A2000 vs RTX 4000
+• Costo real: cloud vs edge Bogotá
+• Casos reales: bodega, centro logístico, farmacias</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1140,6 +1339,16 @@
           <t>https://serviciosapc.site/blog/bot-whatsapp-ia-atencion-clientes-seguridad-bogota</t>
         </is>
       </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Problema: mensajes WhatsApp saturados
+• Qué es Bot WhatsApp con IA vs chatbot tradicional
+• Arquitectura técnica: n8n + GPT + Meta API
+• Flujo detallado con ejemplo real
+• Integración con CCTV y alertas automáticas
+• Caso real: Distribuidora Jone 80% automatización</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1175,6 +1384,17 @@
           <t>https://serviciosapc.site/blog/deteccion-ppe-ia-construccion-fabrica-bogota-cumplimiento</t>
         </is>
       </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Problema: EPP manualmente imposible
+• Qué detecta la IA: casco, chaleco, guantes, gafas
+• Marco normativo SG-SST Colombia
+• Arquitectura del sistema IA en edge
+• DeepinView vs YOLO edge comparativa
+• Caso real: fábrica Ciudad Bolívar
+• Resultados: 0 accidentes, 0 multas, payback 5 meses</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1210,6 +1430,17 @@
           <t>https://serviciosapc.site/blog/hikvision-vs-dahua-vs-uniview-comparativa-ia-2026</t>
         </is>
       </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Qué es cada marca: Hikvision, Dahua, Uniview
+• Tabla comparativa completa 2026
+• Capacidades IA profundidad por marca
+• Precios estimados Colombia 2026
+• Compatibilidad YOLO y análisis externo
+• Visión nocturna comparativa real
+• Casos reales Bogotá por marca</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1245,6 +1476,17 @@
           <t>https://serviciosapc.site/blog/cuanto-cuesta-camaras-seguridad-negocio-bogota-2026</t>
         </is>
       </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Problema: por qué es tan difícil cotizar
+• Qué incluye realmente un sistema CCTV
+• Desglose precios reales Bogotá 2026
+• Escenario 4, 8 y 16 cámaras con y sin IA
+• Costos mensuales recurrentes
+• ROI: cuánto tarda en pagar sola
+• Casos reales: tienda, bodega, restaurante, consultorio</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1280,6 +1522,16 @@
           <t>https://serviciosapc.site/blog/mejores-camaras-seguridad-local-comercial-bogota</t>
         </is>
       </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Problema: elegir cámara incorrecta cuesta más
+• Tipos: bullet, dome, PTZ, fisheye
+• Features clave: resolución, nocturna, IA, PoE
+• Casos reales: cafetería, tienda tech, gimnasio, boutique
+• Guía de compra por tipo de negocio
+• FAQ: cuántas cámaras, Hikvision vs Dahua, DIY</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1315,6 +1567,17 @@
           <t>https://serviciosapc.site/blog/camaras-seguridad-bodega-bogota-monitoreo-inteligente</t>
         </is>
       </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Problema: bodegas como objetivo vulnerable
+• Retos únicos: techos altos, iluminación variable
+• Tecnología IA: YOLO, conteo, heat maps, intrusión
+• Arquitectura sistema CCTV para bodega
+• Automatización n8n: intrusión y control de carga
+• Costos por tamaño de bodega
+• Casos reales: Kennedy, Suba, Engativá</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1348,6 +1611,17 @@
       <c r="G25" s="3" t="inlineStr">
         <is>
           <t>https://serviciosapc.site/blog/instalacion-camaras-seguridad-negocio-pequeno-bogota-guia</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Problema: negocios pequeños instalan mal cámaras
+• Qué necesitas realmente: lista completa
+• Paso a paso instalación profesional
+• Ubicación de cámaras: reglas y errores
+• DIY vs profesional: cuándo contratar
+• Errores comunes y cómo evitarlos
+• Casos reales: tienda, cafetería, taller</t>
         </is>
       </c>
     </row>

</xml_diff>